<commit_message>
fix labour supply loading to pass tests
</commit_message>
<xml_diff>
--- a/input/reg_labourSupplyUtility_UC.xlsx
+++ b/input/reg_labourSupplyUtility_UC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\andy_local\SimPaths project files\SimPaths\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52B508BF-2672-44E9-94D5-23450FCB479F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{596EB9A8-1529-4F96-9E13-6830BE5F8C1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3495" yWindow="3945" windowWidth="21600" windowHeight="11295" activeTab="1" xr2:uid="{DAE320C9-B4E2-7F4A-B376-6CFA80FFD548}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="7" xr2:uid="{DAE320C9-B4E2-7F4A-B376-6CFA80FFD548}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>
@@ -19,8 +19,8 @@
     <sheet name="UK_Couples" sheetId="4" r:id="rId4"/>
     <sheet name="UK_Females_With_Dep" sheetId="5" r:id="rId5"/>
     <sheet name="UK_Males_With_Dep" sheetId="6" r:id="rId6"/>
-    <sheet name="UK_SingleAC_Females" sheetId="7" r:id="rId7"/>
-    <sheet name="UK_SingleAC_Males" sheetId="8" r:id="rId8"/>
+    <sheet name="UK_SingleAC_Females" sheetId="9" r:id="rId7"/>
+    <sheet name="UK_SingleAC_Males" sheetId="10" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="586" uniqueCount="232">
   <si>
     <t>Description:</t>
   </si>
@@ -690,34 +690,7 @@
     <t>MaleIncomeSqDiv10000</t>
   </si>
   <si>
-    <t>FixedCost_Female</t>
-  </si>
-  <si>
     <t>Liwwh_1</t>
-  </si>
-  <si>
-    <t>Liwwh_10</t>
-  </si>
-  <si>
-    <t>Liwwh_11</t>
-  </si>
-  <si>
-    <t>Liwwh_20</t>
-  </si>
-  <si>
-    <t>Liwwh_21</t>
-  </si>
-  <si>
-    <t>Liwwh_30</t>
-  </si>
-  <si>
-    <t>Liwwh_31</t>
-  </si>
-  <si>
-    <t>Liwwh_40</t>
-  </si>
-  <si>
-    <t>Liwwh_41</t>
   </si>
   <si>
     <t>Liwwh_100</t>
@@ -742,6 +715,30 @@
   </si>
   <si>
     <t>Liwwh_401</t>
+  </si>
+  <si>
+    <t>Liwwh_010</t>
+  </si>
+  <si>
+    <t>Liwwh_011</t>
+  </si>
+  <si>
+    <t>Liwwh_020</t>
+  </si>
+  <si>
+    <t>Liwwh_021</t>
+  </si>
+  <si>
+    <t>Liwwh_030</t>
+  </si>
+  <si>
+    <t>Liwwh_031</t>
+  </si>
+  <si>
+    <t>Liwwh_040</t>
+  </si>
+  <si>
+    <t>Liwwh_041</t>
   </si>
 </sst>
 </file>
@@ -63282,7 +63279,7 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{97529604-3295-416D-B8BD-BE16D551132F}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F054EE9D-F9D7-454C-9EEA-D6F644E2F26B}">
   <dimension ref="A1:AE30"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -63330,58 +63327,58 @@
         <v>128</v>
       </c>
       <c r="N1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="O1" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="X1" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="AA1" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="AD1" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
         <v>223</v>
-      </c>
-      <c r="W1" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="X1" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="Y1" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="Z1" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="AA1" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="AB1" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="AC1" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="AD1" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="AE1" s="2" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.25">
@@ -64526,7 +64523,7 @@
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B14" s="2">
         <v>-1.35734328536476E-2</v>
@@ -64621,7 +64618,7 @@
     </row>
     <row r="15" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="B15" s="2">
         <v>-2.0050798941757802E-3</v>
@@ -64716,7 +64713,7 @@
     </row>
     <row r="16" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="B16" s="2">
         <v>-2.2808771051673199E-2</v>
@@ -64811,7 +64808,7 @@
     </row>
     <row r="17" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="B17" s="2">
         <v>1.5803642417603601E-2</v>
@@ -64906,7 +64903,7 @@
     </row>
     <row r="18" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="B18" s="2">
         <v>9.9177244178018896E-3</v>
@@ -65001,7 +64998,7 @@
     </row>
     <row r="19" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="B19" s="2">
         <v>2.2488293912465498E-2</v>
@@ -65096,7 +65093,7 @@
     </row>
     <row r="20" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="B20" s="2">
         <v>1.28100266221424E-2</v>
@@ -65191,7 +65188,7 @@
     </row>
     <row r="21" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="B21" s="2">
         <v>1.7396586469329098E-2</v>
@@ -65286,7 +65283,7 @@
     </row>
     <row r="22" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="B22" s="2">
         <v>-5.54366381774049</v>
@@ -65381,7 +65378,7 @@
     </row>
     <row r="23" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="B23" s="2">
         <v>-1.53561020646784E-2</v>
@@ -65476,7 +65473,7 @@
     </row>
     <row r="24" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="B24" s="2">
         <v>-3.7360726666322598E-2</v>
@@ -65571,7 +65568,7 @@
     </row>
     <row r="25" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="B25" s="2">
         <v>3.57891790059023E-3</v>
@@ -65666,7 +65663,7 @@
     </row>
     <row r="26" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="B26" s="2">
         <v>-10.3024581492006</v>
@@ -65761,7 +65758,7 @@
     </row>
     <row r="27" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="B27" s="2">
         <v>1.3622042802456401E-2</v>
@@ -65856,7 +65853,7 @@
     </row>
     <row r="28" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="B28" s="2">
         <v>-10.6084327042271</v>
@@ -65951,7 +65948,7 @@
     </row>
     <row r="29" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="B29" s="2">
         <v>1.7355003996953899E-2</v>
@@ -66046,7 +66043,7 @@
     </row>
     <row r="30" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="B30" s="2">
         <v>-0.145958808742086</v>
@@ -66141,12 +66138,12 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA73B810-A2AD-4E3D-BEEF-4B6C47FE4F2A}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E18B2A55-65FC-4BCE-86ED-D4BD1F068B09}">
   <dimension ref="A1:AE30"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -66194,58 +66191,58 @@
         <v>128</v>
       </c>
       <c r="N1" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="O1" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="P1" s="2" t="s">
+        <v>224</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>226</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>227</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>228</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>229</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>230</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>231</v>
+      </c>
+      <c r="X1" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="P1" s="2" t="s">
+      <c r="Y1" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="Q1" s="2" t="s">
+      <c r="Z1" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="AA1" s="2" t="s">
         <v>219</v>
       </c>
-      <c r="S1" s="2" t="s">
+      <c r="AB1" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="T1" s="2" t="s">
+      <c r="AC1" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="AD1" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="V1" s="2" t="s">
+      <c r="AE1" s="2" t="s">
         <v>223</v>
-      </c>
-      <c r="W1" s="2" t="s">
-        <v>224</v>
-      </c>
-      <c r="X1" s="2" t="s">
-        <v>225</v>
-      </c>
-      <c r="Y1" s="2" t="s">
-        <v>226</v>
-      </c>
-      <c r="Z1" s="2" t="s">
-        <v>227</v>
-      </c>
-      <c r="AA1" s="2" t="s">
-        <v>228</v>
-      </c>
-      <c r="AB1" s="2" t="s">
-        <v>229</v>
-      </c>
-      <c r="AC1" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="AD1" s="2" t="s">
-        <v>231</v>
-      </c>
-      <c r="AE1" s="2" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="2" spans="1:31" x14ac:dyDescent="0.25">
@@ -67390,7 +67387,7 @@
     </row>
     <row r="14" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B14" s="2">
         <v>-1.35734328536476E-2</v>
@@ -67485,7 +67482,7 @@
     </row>
     <row r="15" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="B15" s="2">
         <v>-2.0050798941757802E-3</v>
@@ -67580,7 +67577,7 @@
     </row>
     <row r="16" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="B16" s="2">
         <v>-2.2808771051673199E-2</v>
@@ -67675,7 +67672,7 @@
     </row>
     <row r="17" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="B17" s="2">
         <v>1.5803642417603601E-2</v>
@@ -67770,7 +67767,7 @@
     </row>
     <row r="18" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="B18" s="2">
         <v>9.9177244178018896E-3</v>
@@ -67865,7 +67862,7 @@
     </row>
     <row r="19" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="B19" s="2">
         <v>2.2488293912465498E-2</v>
@@ -67960,7 +67957,7 @@
     </row>
     <row r="20" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
       <c r="B20" s="2">
         <v>1.28100266221424E-2</v>
@@ -68055,7 +68052,7 @@
     </row>
     <row r="21" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="B21" s="2">
         <v>1.7396586469329098E-2</v>
@@ -68150,7 +68147,7 @@
     </row>
     <row r="22" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="B22" s="2">
         <v>-5.54366381774049</v>
@@ -68245,7 +68242,7 @@
     </row>
     <row r="23" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="B23" s="2">
         <v>-1.53561020646784E-2</v>
@@ -68340,7 +68337,7 @@
     </row>
     <row r="24" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="B24" s="2">
         <v>-3.7360726666322598E-2</v>
@@ -68435,7 +68432,7 @@
     </row>
     <row r="25" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="B25" s="2">
         <v>3.57891790059023E-3</v>
@@ -68530,7 +68527,7 @@
     </row>
     <row r="26" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="B26" s="2">
         <v>-10.3024581492006</v>
@@ -68625,7 +68622,7 @@
     </row>
     <row r="27" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>229</v>
+        <v>220</v>
       </c>
       <c r="B27" s="2">
         <v>1.3622042802456401E-2</v>
@@ -68720,7 +68717,7 @@
     </row>
     <row r="28" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>230</v>
+        <v>221</v>
       </c>
       <c r="B28" s="2">
         <v>-10.6084327042271</v>
@@ -68815,7 +68812,7 @@
     </row>
     <row r="29" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>231</v>
+        <v>222</v>
       </c>
       <c r="B29" s="2">
         <v>1.7355003996953899E-2</v>
@@ -68910,7 +68907,7 @@
     </row>
     <row r="30" spans="1:31" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="B30" s="2">
         <v>-0.145958808742086</v>

</xml_diff>